<commit_message>
Updated with new species
</commit_message>
<xml_diff>
--- a/data/HGT-inserts_summary.xlsx
+++ b/data/HGT-inserts_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F043B69-87AA-004F-BF74-BF6930801A43}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98395CDD-BB8E-9142-9FF8-D6519929E67D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10840" yWindow="500" windowWidth="16020" windowHeight="16420" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
+    <workbookView xWindow="10840" yWindow="500" windowWidth="16020" windowHeight="16380" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t>Genome</t>
   </si>
@@ -154,6 +154,12 @@
   </si>
   <si>
     <t>20230531 - sent by Kiyoto Maekawa</t>
+  </si>
+  <si>
+    <t>Diploptera punctata</t>
+  </si>
+  <si>
+    <t>GCA_030220185.1 - GenBank</t>
   </si>
 </sst>
 </file>
@@ -176,7 +182,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -204,6 +210,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -235,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -246,6 +258,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -580,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40A815C-EDAC-574C-BA26-EF35C495DFC6}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -765,29 +784,27 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="2">
-        <v>358</v>
-      </c>
+    <row r="13" spans="1:6" ht="17">
+      <c r="A13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13" s="10"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>35</v>
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="C14" s="2">
-        <v>142</v>
+        <v>358</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -795,13 +812,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C15" s="5">
-        <v>732</v>
+        <v>35</v>
+      </c>
+      <c r="C15" s="2">
+        <v>142</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -809,10 +826,10 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="5">
         <v>732</v>
@@ -823,13 +840,13 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" s="2">
-        <v>696</v>
+        <v>12</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" s="5">
+        <v>732</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -837,27 +854,27 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="C18" s="2">
-        <v>616</v>
+        <v>696</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>35</v>
+      <c r="A19" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>39</v>
       </c>
       <c r="C19" s="2">
-        <v>4</v>
+        <v>616</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -865,13 +882,13 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>42</v>
+        <v>34</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>35</v>
       </c>
       <c r="C20" s="2">
-        <v>89</v>
+        <v>4</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -879,13 +896,13 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B21" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>42</v>
       </c>
       <c r="C21" s="2">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -893,13 +910,13 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C22" s="2">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -907,17 +924,31 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>41</v>
+        <v>6</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>35</v>
       </c>
       <c r="C23" s="2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" s="2">
+        <v>8</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated insert summary and script 3.4
</commit_message>
<xml_diff>
--- a/data/HGT-inserts_summary.xlsx
+++ b/data/HGT-inserts_summary.xlsx
@@ -1,24 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kewart/Documents/GitHub/HGT_pipeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69CBDBC3-1CFD-AC40-B2BF-3F6AA87D9D6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B531E389-2237-5D49-870B-34291B061D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9780" yWindow="880" windowWidth="22260" windowHeight="16380" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
+    <workbookView xWindow="820" yWindow="1560" windowWidth="20620" windowHeight="16380" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -253,7 +263,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -328,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -344,8 +354,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -680,8 +688,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40A815C-EDAC-574C-BA26-EF35C495DFC6}">
-  <dimension ref="A1:U51"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
+  <dimension ref="A1:U24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="52.33203125" customWidth="1"/>
@@ -691,7 +699,7 @@
     <col min="6" max="21" width="21.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
@@ -756,7 +764,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -786,14 +794,22 @@
       <c r="O2" s="2">
         <v>1849</v>
       </c>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
+      <c r="P2" s="2">
+        <v>1588</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>1575</v>
+      </c>
+      <c r="R2" s="2">
+        <v>1849</v>
+      </c>
+      <c r="S2" s="2">
+        <v>1802</v>
+      </c>
       <c r="T2" s="2"/>
       <c r="U2" s="2"/>
     </row>
-    <row r="3" spans="1:21">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -823,14 +839,22 @@
       <c r="O3" s="2">
         <v>3414</v>
       </c>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
+      <c r="P3" s="2">
+        <v>2920</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>2845</v>
+      </c>
+      <c r="R3" s="2">
+        <v>3414</v>
+      </c>
+      <c r="S3" s="2">
+        <v>3283</v>
+      </c>
       <c r="T3" s="2"/>
       <c r="U3" s="2"/>
     </row>
-    <row r="4" spans="1:21">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -860,14 +884,22 @@
       <c r="O4" s="2">
         <v>5841</v>
       </c>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
+      <c r="P4" s="2">
+        <v>4955</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>4900</v>
+      </c>
+      <c r="R4" s="2">
+        <v>5841</v>
+      </c>
+      <c r="S4" s="2">
+        <v>5669</v>
+      </c>
       <c r="T4" s="2"/>
       <c r="U4" s="2"/>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -897,14 +929,22 @@
       <c r="O5" s="2">
         <v>4865</v>
       </c>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
+      <c r="P5" s="2">
+        <v>4193</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>4117</v>
+      </c>
+      <c r="R5" s="2">
+        <v>4865</v>
+      </c>
+      <c r="S5" s="2">
+        <v>4680</v>
+      </c>
       <c r="T5" s="2"/>
       <c r="U5" s="2"/>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -934,14 +974,22 @@
       <c r="O6" s="2">
         <v>4378</v>
       </c>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
+      <c r="P6" s="2">
+        <v>3794</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>3766</v>
+      </c>
+      <c r="R6" s="2">
+        <v>4378</v>
+      </c>
+      <c r="S6" s="2">
+        <v>4261</v>
+      </c>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -971,14 +1019,22 @@
       <c r="O7" s="2">
         <v>4248</v>
       </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
+      <c r="P7" s="2">
+        <v>3673</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>3637</v>
+      </c>
+      <c r="R7" s="2">
+        <v>4248</v>
+      </c>
+      <c r="S7" s="2">
+        <v>4132</v>
+      </c>
       <c r="T7" s="2"/>
       <c r="U7" s="2"/>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1008,14 +1064,22 @@
       <c r="O8" s="2">
         <v>4621</v>
       </c>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
+      <c r="P8" s="2">
+        <v>4031</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>3926</v>
+      </c>
+      <c r="R8" s="2">
+        <v>4621</v>
+      </c>
+      <c r="S8" s="2">
+        <v>4492</v>
+      </c>
       <c r="T8" s="2"/>
       <c r="U8" s="2"/>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1045,14 +1109,22 @@
       <c r="O9" s="2">
         <v>5389</v>
       </c>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
+      <c r="P9" s="2">
+        <v>4619</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>4561</v>
+      </c>
+      <c r="R9" s="2">
+        <v>5389</v>
+      </c>
+      <c r="S9" s="2">
+        <v>5260</v>
+      </c>
       <c r="T9" s="2"/>
       <c r="U9" s="2"/>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1082,14 +1154,22 @@
       <c r="O10" s="2">
         <v>1814</v>
       </c>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
+      <c r="P10" s="2">
+        <v>1532</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>1499</v>
+      </c>
+      <c r="R10" s="2">
+        <v>1814</v>
+      </c>
+      <c r="S10" s="2">
+        <v>1741</v>
+      </c>
       <c r="T10" s="2"/>
       <c r="U10" s="2"/>
     </row>
-    <row r="11" spans="1:21">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1119,14 +1199,22 @@
       <c r="O11" s="2">
         <v>3120</v>
       </c>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
+      <c r="P11" s="2">
+        <v>2751</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>2705</v>
+      </c>
+      <c r="R11" s="2">
+        <v>3120</v>
+      </c>
+      <c r="S11" s="2">
+        <v>3056</v>
+      </c>
       <c r="T11" s="2"/>
       <c r="U11" s="2"/>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -1156,14 +1244,22 @@
       <c r="O12" s="2">
         <v>4822</v>
       </c>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
+      <c r="P12" s="2">
+        <v>4257</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>4226</v>
+      </c>
+      <c r="R12" s="2">
+        <v>4822</v>
+      </c>
+      <c r="S12" s="2">
+        <v>4690</v>
+      </c>
       <c r="T12" s="2"/>
       <c r="U12" s="2"/>
     </row>
-    <row r="13" spans="1:21" ht="17">
+    <row r="13" spans="1:21" ht="17" x14ac:dyDescent="0.2">
       <c r="A13" s="7" t="s">
         <v>25</v>
       </c>
@@ -1193,14 +1289,22 @@
       <c r="O13" s="2">
         <v>875</v>
       </c>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
+      <c r="P13" s="2">
+        <v>511</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>506</v>
+      </c>
+      <c r="R13" s="2">
+        <v>875</v>
+      </c>
+      <c r="S13" s="2">
+        <v>839</v>
+      </c>
       <c r="T13" s="2"/>
       <c r="U13" s="2"/>
     </row>
-    <row r="14" spans="1:21" ht="17">
+    <row r="14" spans="1:21" ht="17" x14ac:dyDescent="0.2">
       <c r="A14" s="6" t="s">
         <v>11</v>
       </c>
@@ -1230,14 +1334,22 @@
       <c r="O14" s="2">
         <v>466</v>
       </c>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
+      <c r="P14" s="2">
+        <v>308</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>288</v>
+      </c>
+      <c r="R14" s="2">
+        <v>466</v>
+      </c>
+      <c r="S14" s="2">
+        <v>424</v>
+      </c>
       <c r="T14" s="2"/>
       <c r="U14" s="2"/>
     </row>
-    <row r="15" spans="1:21">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
@@ -1267,14 +1379,22 @@
       <c r="O15" s="2">
         <v>246</v>
       </c>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+      <c r="P15" s="2">
+        <v>101</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>93</v>
+      </c>
+      <c r="R15" s="2">
+        <v>246</v>
+      </c>
+      <c r="S15" s="2">
+        <v>226</v>
+      </c>
       <c r="T15" s="2"/>
       <c r="U15" s="2"/>
     </row>
-    <row r="16" spans="1:21">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
@@ -1304,14 +1424,22 @@
       <c r="O16" s="2">
         <v>840</v>
       </c>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
+      <c r="P16" s="2">
+        <v>658</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>644</v>
+      </c>
+      <c r="R16" s="2">
+        <v>840</v>
+      </c>
+      <c r="S16" s="2">
+        <v>793</v>
+      </c>
       <c r="T16" s="2"/>
       <c r="U16" s="2"/>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
@@ -1341,14 +1469,22 @@
       <c r="O17" s="2">
         <v>794</v>
       </c>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
+      <c r="P17" s="2">
+        <v>648</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>639</v>
+      </c>
+      <c r="R17" s="2">
+        <v>794</v>
+      </c>
+      <c r="S17" s="2">
+        <v>781</v>
+      </c>
       <c r="T17" s="2"/>
       <c r="U17" s="2"/>
     </row>
-    <row r="18" spans="1:21">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" s="6" t="s">
         <v>17</v>
       </c>
@@ -1378,14 +1514,22 @@
       <c r="O18" s="2">
         <v>543</v>
       </c>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
+      <c r="P18" s="2">
+        <v>278</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>277</v>
+      </c>
+      <c r="R18" s="2">
+        <v>543</v>
+      </c>
+      <c r="S18" s="2">
+        <v>517</v>
+      </c>
       <c r="T18" s="2"/>
       <c r="U18" s="2"/>
     </row>
-    <row r="19" spans="1:21">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" s="6" t="s">
         <v>8</v>
       </c>
@@ -1415,14 +1559,22 @@
       <c r="O19" s="2">
         <v>555</v>
       </c>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
+      <c r="P19" s="2">
+        <v>285</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>280</v>
+      </c>
+      <c r="R19" s="2">
+        <v>555</v>
+      </c>
+      <c r="S19" s="2">
+        <v>526</v>
+      </c>
       <c r="T19" s="2"/>
       <c r="U19" s="2"/>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
         <v>20</v>
       </c>
@@ -1452,14 +1604,22 @@
       <c r="O20" s="2">
         <v>2</v>
       </c>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
+      <c r="P20" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>0</v>
+      </c>
+      <c r="R20" s="2">
+        <v>2</v>
+      </c>
+      <c r="S20" s="2">
+        <v>2</v>
+      </c>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
     </row>
-    <row r="21" spans="1:21">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
         <v>22</v>
       </c>
@@ -1489,14 +1649,22 @@
       <c r="O21" s="2">
         <v>50</v>
       </c>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
+      <c r="P21" s="2">
+        <v>14</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>14</v>
+      </c>
+      <c r="R21" s="2">
+        <v>50</v>
+      </c>
+      <c r="S21" s="2">
+        <v>42</v>
+      </c>
       <c r="T21" s="2"/>
       <c r="U21" s="2"/>
     </row>
-    <row r="22" spans="1:21">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
@@ -1526,14 +1694,22 @@
       <c r="O22" s="2">
         <v>6</v>
       </c>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="2"/>
-      <c r="S22" s="2"/>
+      <c r="P22" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>0</v>
+      </c>
+      <c r="R22" s="2">
+        <v>6</v>
+      </c>
+      <c r="S22" s="2">
+        <v>6</v>
+      </c>
       <c r="T22" s="2"/>
       <c r="U22" s="2"/>
     </row>
-    <row r="23" spans="1:21">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
         <v>4</v>
       </c>
@@ -1563,14 +1739,22 @@
       <c r="O23" s="2">
         <v>9</v>
       </c>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="2"/>
-      <c r="S23" s="2"/>
+      <c r="P23" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2">
+        <v>9</v>
+      </c>
+      <c r="S23" s="2">
+        <v>9</v>
+      </c>
       <c r="T23" s="2"/>
       <c r="U23" s="2"/>
     </row>
-    <row r="24" spans="1:21">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>24</v>
       </c>
@@ -1588,124 +1772,32 @@
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
-      <c r="L24" s="9">
+      <c r="L24" s="2">
         <v>7</v>
       </c>
       <c r="M24" s="2">
         <v>46</v>
       </c>
-      <c r="N24" s="9">
+      <c r="N24" s="2">
         <v>7</v>
       </c>
       <c r="O24" s="2">
         <v>46</v>
       </c>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
+      <c r="P24" s="2">
+        <v>7</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>7</v>
+      </c>
+      <c r="R24" s="2">
+        <v>46</v>
+      </c>
+      <c r="S24" s="2">
+        <v>46</v>
+      </c>
       <c r="T24" s="2"/>
       <c r="U24" s="2"/>
-    </row>
-    <row r="27" spans="1:21">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-    </row>
-    <row r="28" spans="1:21">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-    </row>
-    <row r="29" spans="1:21">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-    </row>
-    <row r="30" spans="1:21">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-    </row>
-    <row r="31" spans="1:21">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-    </row>
-    <row r="32" spans="1:21">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-    </row>
-    <row r="33" spans="1:2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-    </row>
-    <row r="34" spans="1:2">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-    </row>
-    <row r="35" spans="1:2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="10"/>
-    </row>
-    <row r="36" spans="1:2">
-      <c r="A36" s="10"/>
-      <c r="B36" s="10"/>
-    </row>
-    <row r="37" spans="1:2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="10"/>
-    </row>
-    <row r="38" spans="1:2">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-    </row>
-    <row r="39" spans="1:2">
-      <c r="A39" s="10"/>
-      <c r="B39" s="10"/>
-    </row>
-    <row r="40" spans="1:2">
-      <c r="A40" s="10"/>
-      <c r="B40" s="10"/>
-    </row>
-    <row r="41" spans="1:2">
-      <c r="A41" s="10"/>
-      <c r="B41" s="10"/>
-    </row>
-    <row r="42" spans="1:2">
-      <c r="A42" s="10"/>
-      <c r="B42" s="10"/>
-    </row>
-    <row r="43" spans="1:2">
-      <c r="A43" s="10"/>
-      <c r="B43" s="10"/>
-    </row>
-    <row r="44" spans="1:2">
-      <c r="A44" s="10"/>
-      <c r="B44" s="10"/>
-    </row>
-    <row r="45" spans="1:2">
-      <c r="A45" s="10"/>
-      <c r="B45" s="10"/>
-    </row>
-    <row r="46" spans="1:2">
-      <c r="A46" s="10"/>
-      <c r="B46" s="10"/>
-    </row>
-    <row r="47" spans="1:2">
-      <c r="A47" s="10"/>
-      <c r="B47" s="10"/>
-    </row>
-    <row r="48" spans="1:2">
-      <c r="A48" s="10"/>
-      <c r="B48" s="10"/>
-    </row>
-    <row r="49" spans="1:2">
-      <c r="A49" s="10"/>
-      <c r="B49" s="10"/>
-    </row>
-    <row r="50" spans="1:2">
-      <c r="A50" s="10"/>
-      <c r="B50" s="10"/>
-    </row>
-    <row r="51" spans="1:2">
-      <c r="A51" s="10"/>
-      <c r="B51" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated manuscript and data
</commit_message>
<xml_diff>
--- a/data/HGT-inserts_summary.xlsx
+++ b/data/HGT-inserts_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyleewart/Documents/PostDoc/HGT_pipeline/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00C9D54E-FD1F-084C-A4BD-30EBD59F8B2A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49E345FE-D926-1542-8E5F-7D9AB52FF6A7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8780" yWindow="1600" windowWidth="20620" windowHeight="16380" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
+    <workbookView xWindow="3620" yWindow="760" windowWidth="25740" windowHeight="16380" xr2:uid="{3365DD2C-654A-1041-91AD-AF43EE6D7734}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="77">
   <si>
     <t xml:space="preserve">Panesthia cribrata </t>
   </si>
@@ -250,6 +250,12 @@
   </si>
   <si>
     <t>NA</t>
+  </si>
+  <si>
+    <t>7.v1. HGT insert count - audited</t>
+  </si>
+  <si>
+    <t>7.v2. HGT insert count - audited</t>
   </si>
 </sst>
 </file>
@@ -688,7 +694,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C40A815C-EDAC-574C-BA26-EF35C495DFC6}">
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:W24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="46" bestFit="1" customWidth="1"/>
@@ -696,10 +702,14 @@
     <col min="3" max="3" width="51.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.83203125" customWidth="1"/>
     <col min="5" max="5" width="41.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="21" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="16" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="29.83203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="23" width="21.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21">
+    <row r="1" spans="1:23">
       <c r="A1" s="4" t="s">
         <v>33</v>
       </c>
@@ -749,22 +759,28 @@
         <v>68</v>
       </c>
       <c r="Q1" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="R1" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="T1" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="U1" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="T1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:21">
+    <row r="2" spans="1:23">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
@@ -798,22 +814,28 @@
         <v>1588</v>
       </c>
       <c r="Q2" s="2">
+        <v>1588</v>
+      </c>
+      <c r="R2" s="2">
         <v>1575</v>
       </c>
-      <c r="R2" s="2">
+      <c r="S2" s="2">
+        <v>1575</v>
+      </c>
+      <c r="T2" s="2">
         <v>1849</v>
       </c>
-      <c r="S2" s="2">
+      <c r="U2" s="2">
         <v>1802</v>
       </c>
-      <c r="T2" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U2" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21">
+      <c r="V2" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W2" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -847,22 +869,28 @@
         <v>2920</v>
       </c>
       <c r="Q3" s="2">
+        <v>2920</v>
+      </c>
+      <c r="R3" s="2">
         <v>2845</v>
       </c>
-      <c r="R3" s="2">
+      <c r="S3" s="2">
+        <v>2845</v>
+      </c>
+      <c r="T3" s="2">
         <v>3414</v>
       </c>
-      <c r="S3" s="2">
+      <c r="U3" s="2">
         <v>3283</v>
       </c>
-      <c r="T3" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U3" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21">
+      <c r="V3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W3" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -896,22 +924,28 @@
         <v>4955</v>
       </c>
       <c r="Q4" s="2">
+        <v>4955</v>
+      </c>
+      <c r="R4" s="2">
         <v>4900</v>
       </c>
-      <c r="R4" s="2">
+      <c r="S4" s="2">
+        <v>4900</v>
+      </c>
+      <c r="T4" s="2">
         <v>5841</v>
       </c>
-      <c r="S4" s="2">
+      <c r="U4" s="2">
         <v>5669</v>
       </c>
-      <c r="T4" s="2">
+      <c r="V4" s="2">
         <v>626</v>
       </c>
-      <c r="U4" s="2">
+      <c r="W4" s="2">
         <v>784</v>
       </c>
     </row>
-    <row r="5" spans="1:21">
+    <row r="5" spans="1:23">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -945,22 +979,28 @@
         <v>4193</v>
       </c>
       <c r="Q5" s="2">
+        <v>4193</v>
+      </c>
+      <c r="R5" s="2">
         <v>4117</v>
       </c>
-      <c r="R5" s="2">
+      <c r="S5" s="2">
+        <v>4117</v>
+      </c>
+      <c r="T5" s="2">
         <v>4865</v>
       </c>
-      <c r="S5" s="2">
+      <c r="U5" s="2">
         <v>4680</v>
       </c>
-      <c r="T5" s="2">
+      <c r="V5" s="2">
         <v>536</v>
       </c>
-      <c r="U5" s="2">
+      <c r="W5" s="2">
         <v>641</v>
       </c>
     </row>
-    <row r="6" spans="1:21">
+    <row r="6" spans="1:23">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -994,22 +1034,28 @@
         <v>3794</v>
       </c>
       <c r="Q6" s="2">
+        <v>3794</v>
+      </c>
+      <c r="R6" s="2">
         <v>3766</v>
       </c>
-      <c r="R6" s="2">
+      <c r="S6" s="2">
+        <v>3766</v>
+      </c>
+      <c r="T6" s="2">
         <v>4378</v>
       </c>
-      <c r="S6" s="2">
+      <c r="U6" s="2">
         <v>4261</v>
       </c>
-      <c r="T6" s="2">
+      <c r="V6" s="2">
         <v>726</v>
       </c>
-      <c r="U6" s="2">
+      <c r="W6" s="2">
         <v>841</v>
       </c>
     </row>
-    <row r="7" spans="1:21">
+    <row r="7" spans="1:23">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1043,22 +1089,28 @@
         <v>3673</v>
       </c>
       <c r="Q7" s="2">
+        <v>3673</v>
+      </c>
+      <c r="R7" s="2">
         <v>3637</v>
       </c>
-      <c r="R7" s="2">
+      <c r="S7" s="2">
+        <v>3637</v>
+      </c>
+      <c r="T7" s="2">
         <v>4248</v>
       </c>
-      <c r="S7" s="2">
+      <c r="U7" s="2">
         <v>4132</v>
       </c>
-      <c r="T7" s="2">
+      <c r="V7" s="2">
         <v>591</v>
       </c>
-      <c r="U7" s="2">
+      <c r="W7" s="2">
         <v>703</v>
       </c>
     </row>
-    <row r="8" spans="1:21">
+    <row r="8" spans="1:23">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1092,22 +1144,28 @@
         <v>4031</v>
       </c>
       <c r="Q8" s="2">
+        <v>4031</v>
+      </c>
+      <c r="R8" s="2">
         <v>3926</v>
       </c>
-      <c r="R8" s="2">
+      <c r="S8" s="2">
+        <v>3926</v>
+      </c>
+      <c r="T8" s="2">
         <v>4621</v>
       </c>
-      <c r="S8" s="2">
+      <c r="U8" s="2">
         <v>4492</v>
       </c>
-      <c r="T8" s="2">
+      <c r="V8" s="2">
         <v>464</v>
       </c>
-      <c r="U8" s="2">
+      <c r="W8" s="2">
         <v>593</v>
       </c>
     </row>
-    <row r="9" spans="1:21">
+    <row r="9" spans="1:23">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1141,22 +1199,28 @@
         <v>4619</v>
       </c>
       <c r="Q9" s="2">
+        <v>4619</v>
+      </c>
+      <c r="R9" s="2">
         <v>4561</v>
       </c>
-      <c r="R9" s="2">
+      <c r="S9" s="2">
+        <v>4561</v>
+      </c>
+      <c r="T9" s="2">
         <v>5389</v>
       </c>
-      <c r="S9" s="2">
+      <c r="U9" s="2">
         <v>5260</v>
       </c>
-      <c r="T9" s="2">
+      <c r="V9" s="2">
         <v>652</v>
       </c>
-      <c r="U9" s="2">
+      <c r="W9" s="2">
         <v>794</v>
       </c>
     </row>
-    <row r="10" spans="1:21">
+    <row r="10" spans="1:23">
       <c r="A10" s="1" t="s">
         <v>0</v>
       </c>
@@ -1190,22 +1254,28 @@
         <v>1532</v>
       </c>
       <c r="Q10" s="2">
+        <v>1532</v>
+      </c>
+      <c r="R10" s="2">
         <v>1499</v>
       </c>
-      <c r="R10" s="2">
+      <c r="S10" s="2">
+        <v>1499</v>
+      </c>
+      <c r="T10" s="2">
         <v>1814</v>
       </c>
-      <c r="S10" s="2">
+      <c r="U10" s="2">
         <v>1741</v>
       </c>
-      <c r="T10" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U10" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21">
+      <c r="V10" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W10" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1239,22 +1309,28 @@
         <v>2751</v>
       </c>
       <c r="Q11" s="2">
+        <v>2751</v>
+      </c>
+      <c r="R11" s="2">
         <v>2705</v>
       </c>
-      <c r="R11" s="2">
+      <c r="S11" s="2">
+        <v>2705</v>
+      </c>
+      <c r="T11" s="2">
         <v>3120</v>
       </c>
-      <c r="S11" s="2">
+      <c r="U11" s="2">
         <v>3056</v>
       </c>
-      <c r="T11" s="2">
+      <c r="V11" s="2">
         <v>573</v>
       </c>
-      <c r="U11" s="2">
+      <c r="W11" s="2">
         <v>656</v>
       </c>
     </row>
-    <row r="12" spans="1:21">
+    <row r="12" spans="1:23">
       <c r="A12" s="1" t="s">
         <v>18</v>
       </c>
@@ -1288,22 +1364,28 @@
         <v>4257</v>
       </c>
       <c r="Q12" s="2">
+        <v>4257</v>
+      </c>
+      <c r="R12" s="2">
         <v>4226</v>
       </c>
-      <c r="R12" s="2">
+      <c r="S12" s="2">
+        <v>4226</v>
+      </c>
+      <c r="T12" s="2">
         <v>4822</v>
       </c>
-      <c r="S12" s="2">
+      <c r="U12" s="2">
         <v>4690</v>
       </c>
-      <c r="T12" s="2">
+      <c r="V12" s="2">
         <v>616</v>
       </c>
-      <c r="U12" s="2">
+      <c r="W12" s="2">
         <v>719</v>
       </c>
     </row>
-    <row r="13" spans="1:21" ht="17">
+    <row r="13" spans="1:23" ht="17">
       <c r="A13" s="7" t="s">
         <v>25</v>
       </c>
@@ -1337,22 +1419,28 @@
         <v>511</v>
       </c>
       <c r="Q13" s="2">
+        <v>511</v>
+      </c>
+      <c r="R13" s="2">
         <v>506</v>
       </c>
-      <c r="R13" s="2">
+      <c r="S13" s="2">
+        <v>506</v>
+      </c>
+      <c r="T13" s="2">
         <v>875</v>
       </c>
-      <c r="S13" s="2">
+      <c r="U13" s="2">
         <v>839</v>
       </c>
-      <c r="T13" s="2">
+      <c r="V13" s="2">
         <v>19</v>
       </c>
-      <c r="U13" s="2">
+      <c r="W13" s="2">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:21" ht="17">
+    <row r="14" spans="1:23" ht="17">
       <c r="A14" s="6" t="s">
         <v>11</v>
       </c>
@@ -1386,22 +1474,28 @@
         <v>308</v>
       </c>
       <c r="Q14" s="2">
+        <v>308</v>
+      </c>
+      <c r="R14" s="2">
         <v>288</v>
       </c>
-      <c r="R14" s="2">
+      <c r="S14" s="2">
+        <v>288</v>
+      </c>
+      <c r="T14" s="2">
         <v>466</v>
       </c>
-      <c r="S14" s="2">
+      <c r="U14" s="2">
         <v>424</v>
       </c>
-      <c r="T14" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U14" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21">
+      <c r="V14" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W14" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23">
       <c r="A15" s="6" t="s">
         <v>7</v>
       </c>
@@ -1435,22 +1529,28 @@
         <v>101</v>
       </c>
       <c r="Q15" s="2">
+        <v>101</v>
+      </c>
+      <c r="R15" s="2">
         <v>93</v>
       </c>
-      <c r="R15" s="2">
+      <c r="S15" s="2">
+        <v>93</v>
+      </c>
+      <c r="T15" s="2">
         <v>246</v>
       </c>
-      <c r="S15" s="2">
+      <c r="U15" s="2">
         <v>226</v>
       </c>
-      <c r="T15" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U15" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21">
+      <c r="V15" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W15" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
@@ -1484,22 +1584,28 @@
         <v>658</v>
       </c>
       <c r="Q16" s="2">
+        <v>658</v>
+      </c>
+      <c r="R16" s="2">
         <v>644</v>
       </c>
-      <c r="R16" s="2">
+      <c r="S16" s="2">
+        <v>644</v>
+      </c>
+      <c r="T16" s="2">
         <v>840</v>
       </c>
-      <c r="S16" s="2">
+      <c r="U16" s="2">
         <v>793</v>
       </c>
-      <c r="T16" s="2">
+      <c r="V16" s="2">
         <v>2</v>
       </c>
-      <c r="U16" s="2">
+      <c r="W16" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:21">
+    <row r="17" spans="1:23">
       <c r="A17" s="6" t="s">
         <v>10</v>
       </c>
@@ -1533,22 +1639,28 @@
         <v>648</v>
       </c>
       <c r="Q17" s="2">
+        <v>648</v>
+      </c>
+      <c r="R17" s="2">
         <v>639</v>
       </c>
-      <c r="R17" s="2">
+      <c r="S17" s="2">
+        <v>639</v>
+      </c>
+      <c r="T17" s="2">
         <v>794</v>
       </c>
-      <c r="S17" s="2">
+      <c r="U17" s="2">
         <v>781</v>
       </c>
-      <c r="T17" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U17" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21">
+      <c r="V17" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W17" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23">
       <c r="A18" s="6" t="s">
         <v>17</v>
       </c>
@@ -1582,22 +1694,28 @@
         <v>278</v>
       </c>
       <c r="Q18" s="2">
+        <v>278</v>
+      </c>
+      <c r="R18" s="2">
         <v>277</v>
       </c>
-      <c r="R18" s="2">
+      <c r="S18" s="2">
+        <v>277</v>
+      </c>
+      <c r="T18" s="2">
         <v>543</v>
       </c>
-      <c r="S18" s="2">
+      <c r="U18" s="2">
         <v>517</v>
       </c>
-      <c r="T18" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U18" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21">
+      <c r="V18" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W18" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:23">
       <c r="A19" s="6" t="s">
         <v>8</v>
       </c>
@@ -1631,22 +1749,28 @@
         <v>285</v>
       </c>
       <c r="Q19" s="2">
+        <v>285</v>
+      </c>
+      <c r="R19" s="2">
         <v>280</v>
       </c>
-      <c r="R19" s="2">
+      <c r="S19" s="2">
+        <v>280</v>
+      </c>
+      <c r="T19" s="2">
         <v>555</v>
       </c>
-      <c r="S19" s="2">
+      <c r="U19" s="2">
         <v>526</v>
       </c>
-      <c r="T19" s="2">
+      <c r="V19" s="2">
         <v>7</v>
       </c>
-      <c r="U19" s="2">
+      <c r="W19" s="2">
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:21">
+    <row r="20" spans="1:23">
       <c r="A20" s="3" t="s">
         <v>20</v>
       </c>
@@ -1683,19 +1807,25 @@
         <v>0</v>
       </c>
       <c r="R20" s="2">
+        <v>0</v>
+      </c>
+      <c r="S20" s="2">
+        <v>0</v>
+      </c>
+      <c r="T20" s="2">
         <v>2</v>
       </c>
-      <c r="S20" s="2">
+      <c r="U20" s="2">
         <v>2</v>
       </c>
-      <c r="T20" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U20" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21">
+      <c r="V20" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W20" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23">
       <c r="A21" s="3" t="s">
         <v>22</v>
       </c>
@@ -1729,22 +1859,28 @@
         <v>14</v>
       </c>
       <c r="Q21" s="2">
+        <v>1</v>
+      </c>
+      <c r="R21" s="2">
         <v>14</v>
       </c>
-      <c r="R21" s="2">
+      <c r="S21" s="2">
+        <v>1</v>
+      </c>
+      <c r="T21" s="2">
         <v>50</v>
       </c>
-      <c r="S21" s="2">
+      <c r="U21" s="2">
         <v>42</v>
       </c>
-      <c r="T21" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U21" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21">
+      <c r="V21" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W21" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
@@ -1781,19 +1917,25 @@
         <v>0</v>
       </c>
       <c r="R22" s="2">
+        <v>0</v>
+      </c>
+      <c r="S22" s="2">
+        <v>0</v>
+      </c>
+      <c r="T22" s="2">
         <v>6</v>
       </c>
-      <c r="S22" s="2">
+      <c r="U22" s="2">
         <v>6</v>
       </c>
-      <c r="T22" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U22" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="23" spans="1:21">
+      <c r="V22" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W22" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23">
       <c r="A23" s="3" t="s">
         <v>4</v>
       </c>
@@ -1830,19 +1972,25 @@
         <v>0</v>
       </c>
       <c r="R23" s="2">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2">
+        <v>0</v>
+      </c>
+      <c r="T23" s="2">
         <v>9</v>
       </c>
-      <c r="S23" s="2">
+      <c r="U23" s="2">
         <v>9</v>
       </c>
-      <c r="T23" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U23" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="24" spans="1:21">
+      <c r="V23" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W23" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23">
       <c r="A24" s="3" t="s">
         <v>24</v>
       </c>
@@ -1876,29 +2024,25 @@
         <v>7</v>
       </c>
       <c r="Q24" s="2">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2">
         <v>7</v>
       </c>
-      <c r="R24" s="2">
+      <c r="S24" s="2">
+        <v>0</v>
+      </c>
+      <c r="T24" s="2">
         <v>46</v>
       </c>
-      <c r="S24" s="2">
+      <c r="U24" s="2">
         <v>46</v>
       </c>
-      <c r="T24" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="U24" s="9" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21">
-      <c r="P25">
-        <f>MAX(P2:P24)</f>
-        <v>4955</v>
-      </c>
-      <c r="Q25">
-        <f>MAX(Q2:Q24)</f>
-        <v>4900</v>
+      <c r="V24" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="W24" s="9" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>